<commit_message>
uitbreiding met tweede vergadering
</commit_message>
<xml_diff>
--- a/input/Bestandsbeschrijvingen.xlsx
+++ b/input/Bestandsbeschrijvingen.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ronaldkoenis/eclipse-workspace/maakmdto/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84C75126-A98B-834C-82F8-6C8A92270F50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A026914F-354E-6241-A842-569DB7EC18DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-7560" yWindow="-17500" windowWidth="50640" windowHeight="13120" xr2:uid="{597D6162-B0B0-3844-A8E7-90BC6507AED4}"/>
+    <workbookView xWindow="-16400" yWindow="-28200" windowWidth="51200" windowHeight="20220" xr2:uid="{597D6162-B0B0-3844-A8E7-90BC6507AED4}"/>
   </bookViews>
   <sheets>
     <sheet name="Bestand.zaak en doc" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="576" uniqueCount="280">
   <si>
     <t>Geef per besatnd de zaakgegevens op</t>
   </si>
@@ -671,6 +671,216 @@
   </si>
   <si>
     <t>Behandeling van de programmabegroting 2018</t>
+  </si>
+  <si>
+    <t>2018-03-06/Besluitenlijst-BESL-INT_3346CC83C70245C7A759CEC53465DD8F januari.pdf</t>
+  </si>
+  <si>
+    <t>2018-03-06/Besluitenlijst-BESL-INT_C257092D8760438382D756BBAAFB7F82 februari.pdf</t>
+  </si>
+  <si>
+    <t>2018-03-06/Agenda (gewijzigd) Gemeenteraad_06-03-2018 (20180301).pdf</t>
+  </si>
+  <si>
+    <t>2018-03-06/Lijst ingekomen stukken tm 21 februari 2018.pdf</t>
+  </si>
+  <si>
+    <t>2018-03-06/Lijst ingekomen stukken februari 2018.pdf</t>
+  </si>
+  <si>
+    <t>2018-03-06/7. Bp Landelijk Gebied West - Aanpassing/nr 7 rvs en rbs Bp Landelijk Gebied West 1e herziening - (gewijzigd na cie FD 20180206).pdf</t>
+  </si>
+  <si>
+    <t>2018-03-06/7. Bp Landelijk Gebied West - Aanpassing/Uitspraak Raad van State 20170927 - Bp Landelijk gebied West 1e herziening.pdf</t>
+  </si>
+  <si>
+    <t>2018-03-06/7. Bp Landelijk Gebied West - Aanpassing/Bp Landelijk Gebied West 1e herziening - Regels.pdf</t>
+  </si>
+  <si>
+    <t>2018-03-06/7. Bp Landelijk Gebied West - Aanpassing/Brief fam. Spithoven.pdf</t>
+  </si>
+  <si>
+    <t>2018-03-06/7. Bp Landelijk Gebied West - Aanpassing/Bp Landelijk Gebied West 1e herziening - Verbeelding 20180109 - Overzicht.pdf</t>
+  </si>
+  <si>
+    <t>2018-03-06/7. Bp Landelijk Gebied West - Aanpassing/Bp Landelijk Gebied West 1e herziening - Toelichting.pdf</t>
+  </si>
+  <si>
+    <t>2018-03-06/7. Bp Landelijk Gebied West - Aanpassing/Bp Landelijk Gebied West 1e herziening - Verbeelding 20180109 - Oukoop 22.pdf</t>
+  </si>
+  <si>
+    <t>2018-03-06/8. Bp Landelijk gebied noord - Aanpassing/rvs (gewijzigd) Bp Landelijk gebied noord - Aanpassing.pdf</t>
+  </si>
+  <si>
+    <t>2018-03-06/8. Bp Landelijk gebied noord - Aanpassing/nr 8 rvs en rbs Bp Landelijk gebied noord - Aanpassing.pdf</t>
+  </si>
+  <si>
+    <t>2018-03-06/8. Bp Landelijk gebied noord - Aanpassing/Memo technische wijziging raadsvoorstel Bp Landelijk gebied noord - 20180226.pdf</t>
+  </si>
+  <si>
+    <t>2018-03-06/8. Bp Landelijk gebied noord - Aanpassing/Memo (gewijzigd) technische wijziging raadsvoorstel Bp Landelijk Gebied Noord.pdf</t>
+  </si>
+  <si>
+    <t>2018-03-06/8. Bp Landelijk gebied noord - Aanpassing/rbs (gewijzigd) Bp Landelijk gebied noord - Aanpassing.pdf</t>
+  </si>
+  <si>
+    <t>2018-03-06/9. Bp Beek en Hoff/Nota Zienswijzen Bp Beek en Hoff - gewijzigd n.a.v. commissie FD 6-2-2018 (opm. SVB).pdf</t>
+  </si>
+  <si>
+    <t>2018-03-06/9. Bp Beek en Hoff/Toelichting - Ontwerp Bp Buitenplaats Beek en Hoff.pdf</t>
+  </si>
+  <si>
+    <t>2018-03-06/9. Bp Beek en Hoff/B. Bal - Zienswijze op Bp Buitenplaats Beek en Hoff.pdf</t>
+  </si>
+  <si>
+    <t>2018-03-06/9. Bp Beek en Hoff/Regels - Ontwerp Bp Buitenplaats Beek en Hoff.pdf</t>
+  </si>
+  <si>
+    <t>2018-03-06/9. Bp Beek en Hoff/nr. 9 rvs en rbs Gewijzigd ontwerp Bp Buitenplaats Beek en Hoff.pdf</t>
+  </si>
+  <si>
+    <t>2018-03-06/9. Bp Beek en Hoff/Bijlage 1 - Quickscan Flora en Fauna - Gewijzigd ontwerp Bp Buitenplaats Beek en Hoff.pdf</t>
+  </si>
+  <si>
+    <t>2018-03-06/9. Bp Beek en Hoff/Regels - Gewijzigd ontwerp Bp Buitenplaats Beek en Hoff.pdf</t>
+  </si>
+  <si>
+    <t>2018-03-06/9. Bp Beek en Hoff/Johan Spijker en Margriet Spijker de Wild - Zienswijze op Bp Buitenplaats Beek en Hoff.pdf</t>
+  </si>
+  <si>
+    <t>2018-03-06/9. Bp Beek en Hoff/Regels Bp Beek en Hoff - gewijzigd n.a.v. commissie FD 6-2-2018 (opm. SVB).pdf</t>
+  </si>
+  <si>
+    <t>2018-03-06/9. Bp Beek en Hoff/AKD namens F. Matser zienswijze op Bp Buitenplaats Beek en Hoff.pdf</t>
+  </si>
+  <si>
+    <t>2018-03-06/9. Bp Beek en Hoff/J.E. Spee - Zienswijze op Bp Buitenplaats Beek en Hoff + bijlage.pdf</t>
+  </si>
+  <si>
+    <t>2018-03-06/9. Bp Beek en Hoff/Nota zienswijzen - Gewijzigd ontwerp Bp Buitenplaats Beek en Hoff.pdf</t>
+  </si>
+  <si>
+    <t>2018-03-06/9. Bp Beek en Hoff/N.H.C. van Wijk-Hendrickx e.a. - Zienswijze Bp Buitenplaats Beek en Hoff.pdf</t>
+  </si>
+  <si>
+    <t>2018-03-06/9. Bp Beek en Hoff/Verbeelding - Ontwerp Bp Buitenplaats Beek en Hoff.pdf</t>
+  </si>
+  <si>
+    <t>2018-03-06/9. Bp Beek en Hoff/Toelichting - Gewijzigd ontwerp Bp Buitenplaats Beek en Hoff.pdf</t>
+  </si>
+  <si>
+    <t>2018-03-06/9. Bp Beek en Hoff/Bijlage 2 - Ecologisch onderzoek (dec. 2017) - Gewijzigd ontwerp Bp Buitenplaats Beek en Hoff.pdf</t>
+  </si>
+  <si>
+    <t>2018-03-06/9. Bp Beek en Hoff/Verbeelding - Gewijzigd ontwerp Bp Buitenplaats Beek en Hoff.pdf</t>
+  </si>
+  <si>
+    <t>Raadsvergadering 6 maart 2018</t>
+  </si>
+  <si>
+    <t>Ingekomen stukken</t>
+  </si>
+  <si>
+    <t>Bp Landelijk gebied West - 1e herziening</t>
+  </si>
+  <si>
+    <t>Bp Landelijk gebied noord - Aanpassing</t>
+  </si>
+  <si>
+    <t>Bp Gewijzigd ontwerp Bp Buitenplaats Beek en Hoff</t>
+  </si>
+  <si>
+    <t>Raadsvoorstel en besluit Bestemmingsplan Landelijk Gebied West 1e herziening</t>
+  </si>
+  <si>
+    <t>Uitspraak Raad van State 20170927 - Bp Landelijk gebied West 1e herziening.pdf</t>
+  </si>
+  <si>
+    <t>Brief fam. Spithoven</t>
+  </si>
+  <si>
+    <t>Bp Landelijk Gebied West 1e herziening - Regels</t>
+  </si>
+  <si>
+    <t>Bp Landelijk Gebied West 1e herziening - Verbeelding 20180109 - Overzicht</t>
+  </si>
+  <si>
+    <t>Bp Landelijk Gebied West 1e herziening - Toelichting</t>
+  </si>
+  <si>
+    <t>Bp Landelijk Gebied West 1e herziening - Verbeelding 20180109 - Oukoop 22</t>
+  </si>
+  <si>
+    <t>rvs (gewijzigd) Bp Landelijk gebied noord - Aanpassing</t>
+  </si>
+  <si>
+    <t>Raadsvoorstel en besluit Bestemmingsplan Landelijk gebied noord - Aanpassing</t>
+  </si>
+  <si>
+    <t>Memo technische wijziging raadsvoorstel Bp Landelijk gebied noord - 20180226</t>
+  </si>
+  <si>
+    <t>Memo (gewijzigd) technische wijziging raadsvoorstel Bp Landelijk Gebied Noord</t>
+  </si>
+  <si>
+    <t>rbs (gewijzigd) Bp Landelijk gebied noord - Aanpassing</t>
+  </si>
+  <si>
+    <t>Nota Zienswijzen Bp Beek en Hoff - gewijzigd n.a.v. commissie FD 6-2-2018 (opm. SVB)</t>
+  </si>
+  <si>
+    <t>Toelichting - Ontwerp Bp Buitenplaats Beek en Hoff</t>
+  </si>
+  <si>
+    <t>B. Bal - Zienswijze op Bp Buitenplaats Beek en Hoff</t>
+  </si>
+  <si>
+    <t>Nota zienswijzen (ondertekend) - Gewijzigd ontwerp Bp Buitenplaats Beek en Hoff</t>
+  </si>
+  <si>
+    <t>Regels - Ontwerp Bp Buitenplaats Beek en Hoff</t>
+  </si>
+  <si>
+    <t>Bijlage 1 - Quickscan Flora en Fauna - Gewijzigd ontwerp Bp Buitenplaats Beek en Hoff</t>
+  </si>
+  <si>
+    <t>Regels - Gewijzigd ontwerp Bp Buitenplaats Beek en Hoff</t>
+  </si>
+  <si>
+    <t>Johan Spijker en Margriet Spijker de Wild - Zienswijze op Bp Buitenplaats Beek en Hoff</t>
+  </si>
+  <si>
+    <t>Regels Bp Beek en Hoff - gewijzigd n.a.v. commissie FD 6-2-2018 (opm. SVB)</t>
+  </si>
+  <si>
+    <t>AKD namens F. Matser zienswijze op Bp Buitenplaats Beek en Hoff</t>
+  </si>
+  <si>
+    <t>J.E. Spee - Zienswijze op Bp Buitenplaats Beek en Hoff + bijlage</t>
+  </si>
+  <si>
+    <t>Nota zienswijzen - Gewijzigd ontwerp Bp Buitenplaats Beek en Hoff</t>
+  </si>
+  <si>
+    <t>N.H.C. van Wijk-Hendrickx e.a. - Zienswijze Bp Buitenplaats Beek en Hoff</t>
+  </si>
+  <si>
+    <t>Verbeelding - Ontwerp Bp Buitenplaats Beek en Hoff</t>
+  </si>
+  <si>
+    <t>Toelichting - Gewijzigd ontwerp Bp Buitenplaats Beek en Hoff</t>
+  </si>
+  <si>
+    <t>Bijlage 2 - Ecologisch onderzoek (dec. 2017) - Gewijzigd ontwerp Bp Buitenplaats Beek en Hoff</t>
+  </si>
+  <si>
+    <t>Verbeelding - Gewijzigd ontwerp Bp Buitenplaats Beek en Hoff</t>
+  </si>
+  <si>
+    <t>Raadsvoorstel en besluit Gewijzigd ontwerp Bestemmingsplan Buitenplaats Beek en Hoff</t>
+  </si>
+  <si>
+    <t>2018-03-06/9. Bp Beek en Hoff/Nota zienswijzen (ondertekend)  - Gewijzigd ontwerp Bp Buitenplaats Beek en Hoff.pdf</t>
   </si>
 </sst>
 </file>
@@ -1196,7 +1406,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4C64E42-9F84-ED4B-87CF-18995B18C14B}">
-  <dimension ref="A1:M19"/>
+  <dimension ref="A1:M53"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="140.1640625" customWidth="1"/>
@@ -1207,7 +1417,7 @@
     <col min="8" max="8" width="10.83203125" style="18" customWidth="1"/>
     <col min="9" max="9" width="39.33203125" customWidth="1"/>
     <col min="10" max="10" width="9.83203125" customWidth="1"/>
-    <col min="11" max="11" width="79" customWidth="1"/>
+    <col min="11" max="11" width="111.6640625" customWidth="1"/>
     <col min="12" max="12" width="28.6640625" customWidth="1"/>
     <col min="13" max="13" width="20.83203125" bestFit="1" customWidth="1"/>
   </cols>
@@ -1278,7 +1488,7 @@
       <c r="H2" s="17"/>
       <c r="I2" s="3"/>
       <c r="J2" s="3" t="str">
-        <f t="shared" ref="J2:J18" si="0">C2&amp;"."&amp;ROW()</f>
+        <f t="shared" ref="J2:J53" si="0">C2&amp;"."&amp;ROW()</f>
         <v>1.2</v>
       </c>
       <c r="K2" t="s">
@@ -1944,11 +2154,1379 @@
       <c r="M18" s="2"/>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A19" s="4"/>
+      <c r="A19" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="B19" t="s">
+        <v>3</v>
+      </c>
+      <c r="C19">
+        <v>2</v>
+      </c>
+      <c r="D19" t="s">
+        <v>244</v>
+      </c>
+      <c r="E19" t="s">
+        <v>4</v>
+      </c>
+      <c r="F19" s="2">
+        <v>43165</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="J19" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>2.19</v>
+      </c>
+      <c r="K19" t="s">
+        <v>212</v>
+      </c>
+      <c r="L19" t="s">
+        <v>186</v>
+      </c>
+      <c r="M19" s="2">
+        <v>43165</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A20" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="B20" t="s">
+        <v>3</v>
+      </c>
+      <c r="C20">
+        <v>2</v>
+      </c>
+      <c r="D20" t="s">
+        <v>244</v>
+      </c>
+      <c r="E20" t="s">
+        <v>4</v>
+      </c>
+      <c r="F20" s="2">
+        <v>43165</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="J20" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>2.20</v>
+      </c>
+      <c r="K20" t="s">
+        <v>210</v>
+      </c>
+      <c r="L20" t="s">
+        <v>185</v>
+      </c>
+      <c r="M20" s="2">
+        <v>43165</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A21" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="B21" t="s">
+        <v>3</v>
+      </c>
+      <c r="C21">
+        <v>2</v>
+      </c>
+      <c r="D21" t="s">
+        <v>244</v>
+      </c>
+      <c r="E21" t="s">
+        <v>4</v>
+      </c>
+      <c r="F21" s="2">
+        <v>43165</v>
+      </c>
+      <c r="G21" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="J21" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>2.21</v>
+      </c>
+      <c r="K21" t="s">
+        <v>211</v>
+      </c>
+      <c r="L21" t="s">
+        <v>185</v>
+      </c>
+      <c r="M21" s="2">
+        <v>43165</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A22" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="B22" t="s">
+        <v>3</v>
+      </c>
+      <c r="C22">
+        <v>2</v>
+      </c>
+      <c r="D22" t="s">
+        <v>244</v>
+      </c>
+      <c r="E22" t="s">
+        <v>4</v>
+      </c>
+      <c r="F22" s="2">
+        <v>43165</v>
+      </c>
+      <c r="G22" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H22" s="18">
+        <v>6</v>
+      </c>
+      <c r="I22" t="s">
+        <v>245</v>
+      </c>
+      <c r="J22" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>2.22</v>
+      </c>
+      <c r="K22" t="s">
+        <v>213</v>
+      </c>
+      <c r="L22" t="s">
+        <v>206</v>
+      </c>
+      <c r="M22" s="2">
+        <v>43165</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A23" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="B23" t="s">
+        <v>3</v>
+      </c>
+      <c r="C23">
+        <v>2</v>
+      </c>
+      <c r="D23" t="s">
+        <v>244</v>
+      </c>
+      <c r="E23" t="s">
+        <v>4</v>
+      </c>
+      <c r="F23" s="2">
+        <v>43165</v>
+      </c>
+      <c r="G23" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H23" s="18">
+        <v>6</v>
+      </c>
+      <c r="I23" t="s">
+        <v>245</v>
+      </c>
+      <c r="J23" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>2.23</v>
+      </c>
+      <c r="K23" t="s">
+        <v>214</v>
+      </c>
+      <c r="L23" t="s">
+        <v>206</v>
+      </c>
+      <c r="M23" s="2">
+        <v>43165</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A24" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="B24" t="s">
+        <v>3</v>
+      </c>
+      <c r="C24">
+        <v>2</v>
+      </c>
+      <c r="D24" t="s">
+        <v>244</v>
+      </c>
+      <c r="E24" t="s">
+        <v>4</v>
+      </c>
+      <c r="F24" s="2">
+        <v>43165</v>
+      </c>
+      <c r="G24" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H24" s="18">
+        <v>7</v>
+      </c>
+      <c r="I24" t="s">
+        <v>246</v>
+      </c>
+      <c r="J24" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>2.24</v>
+      </c>
+      <c r="K24" t="s">
+        <v>249</v>
+      </c>
+      <c r="L24" t="s">
+        <v>203</v>
+      </c>
+      <c r="M24" s="2">
+        <v>43165</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A25" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="B25" t="s">
+        <v>3</v>
+      </c>
+      <c r="C25">
+        <v>2</v>
+      </c>
+      <c r="D25" t="s">
+        <v>244</v>
+      </c>
+      <c r="E25" t="s">
+        <v>4</v>
+      </c>
+      <c r="F25" s="2">
+        <v>43165</v>
+      </c>
+      <c r="G25" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H25" s="18">
+        <v>7</v>
+      </c>
+      <c r="I25" t="s">
+        <v>246</v>
+      </c>
+      <c r="J25" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>2.25</v>
+      </c>
+      <c r="K25" t="s">
+        <v>250</v>
+      </c>
+      <c r="L25" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A26" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="B26" t="s">
+        <v>3</v>
+      </c>
+      <c r="C26">
+        <v>2</v>
+      </c>
+      <c r="D26" t="s">
+        <v>244</v>
+      </c>
+      <c r="E26" t="s">
+        <v>4</v>
+      </c>
+      <c r="F26" s="2">
+        <v>43165</v>
+      </c>
+      <c r="G26" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H26" s="18">
+        <v>7</v>
+      </c>
+      <c r="I26" t="s">
+        <v>246</v>
+      </c>
+      <c r="J26" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>2.26</v>
+      </c>
+      <c r="K26" t="s">
+        <v>252</v>
+      </c>
+      <c r="L26" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A27" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="B27" t="s">
+        <v>3</v>
+      </c>
+      <c r="C27">
+        <v>2</v>
+      </c>
+      <c r="D27" t="s">
+        <v>244</v>
+      </c>
+      <c r="E27" t="s">
+        <v>4</v>
+      </c>
+      <c r="F27" s="2">
+        <v>43165</v>
+      </c>
+      <c r="G27" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H27" s="18">
+        <v>7</v>
+      </c>
+      <c r="I27" t="s">
+        <v>246</v>
+      </c>
+      <c r="J27" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>2.27</v>
+      </c>
+      <c r="K27" t="s">
+        <v>251</v>
+      </c>
+      <c r="L27" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A28" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="B28" t="s">
+        <v>3</v>
+      </c>
+      <c r="C28">
+        <v>2</v>
+      </c>
+      <c r="D28" t="s">
+        <v>244</v>
+      </c>
+      <c r="E28" t="s">
+        <v>4</v>
+      </c>
+      <c r="F28" s="2">
+        <v>43165</v>
+      </c>
+      <c r="G28" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H28" s="18">
+        <v>7</v>
+      </c>
+      <c r="I28" t="s">
+        <v>246</v>
+      </c>
+      <c r="J28" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>2.28</v>
+      </c>
+      <c r="K28" t="s">
+        <v>253</v>
+      </c>
+      <c r="L28" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A29" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="B29" t="s">
+        <v>3</v>
+      </c>
+      <c r="C29">
+        <v>2</v>
+      </c>
+      <c r="D29" t="s">
+        <v>244</v>
+      </c>
+      <c r="E29" t="s">
+        <v>4</v>
+      </c>
+      <c r="F29" s="2">
+        <v>43165</v>
+      </c>
+      <c r="G29" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H29" s="18">
+        <v>7</v>
+      </c>
+      <c r="I29" t="s">
+        <v>246</v>
+      </c>
+      <c r="J29" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>2.29</v>
+      </c>
+      <c r="K29" t="s">
+        <v>254</v>
+      </c>
+      <c r="L29" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A30" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="B30" t="s">
+        <v>3</v>
+      </c>
+      <c r="C30">
+        <v>2</v>
+      </c>
+      <c r="D30" t="s">
+        <v>244</v>
+      </c>
+      <c r="E30" t="s">
+        <v>4</v>
+      </c>
+      <c r="F30" s="2">
+        <v>43165</v>
+      </c>
+      <c r="G30" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H30" s="18">
+        <v>7</v>
+      </c>
+      <c r="I30" t="s">
+        <v>246</v>
+      </c>
+      <c r="J30" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>2.30</v>
+      </c>
+      <c r="K30" t="s">
+        <v>255</v>
+      </c>
+      <c r="L30" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A31" s="4" t="s">
+        <v>222</v>
+      </c>
+      <c r="B31" t="s">
+        <v>3</v>
+      </c>
+      <c r="C31">
+        <v>2</v>
+      </c>
+      <c r="D31" t="s">
+        <v>244</v>
+      </c>
+      <c r="E31" t="s">
+        <v>4</v>
+      </c>
+      <c r="F31" s="2">
+        <v>43165</v>
+      </c>
+      <c r="G31" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H31" s="18">
+        <v>8</v>
+      </c>
+      <c r="I31" t="s">
+        <v>247</v>
+      </c>
+      <c r="J31" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>2.31</v>
+      </c>
+      <c r="K31" t="s">
+        <v>256</v>
+      </c>
+      <c r="L31" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A32" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="B32" t="s">
+        <v>3</v>
+      </c>
+      <c r="C32">
+        <v>2</v>
+      </c>
+      <c r="D32" t="s">
+        <v>244</v>
+      </c>
+      <c r="E32" t="s">
+        <v>4</v>
+      </c>
+      <c r="F32" s="2">
+        <v>43165</v>
+      </c>
+      <c r="G32" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H32" s="18">
+        <v>8</v>
+      </c>
+      <c r="I32" t="s">
+        <v>247</v>
+      </c>
+      <c r="J32" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>2.32</v>
+      </c>
+      <c r="K32" t="s">
+        <v>257</v>
+      </c>
+      <c r="L32" t="s">
+        <v>203</v>
+      </c>
+      <c r="M32" s="2">
+        <v>43165</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A33" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="B33" t="s">
+        <v>3</v>
+      </c>
+      <c r="C33">
+        <v>2</v>
+      </c>
+      <c r="D33" t="s">
+        <v>244</v>
+      </c>
+      <c r="E33" t="s">
+        <v>4</v>
+      </c>
+      <c r="F33" s="2">
+        <v>43165</v>
+      </c>
+      <c r="G33" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H33" s="18">
+        <v>8</v>
+      </c>
+      <c r="I33" t="s">
+        <v>247</v>
+      </c>
+      <c r="J33" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>2.33</v>
+      </c>
+      <c r="K33" t="s">
+        <v>258</v>
+      </c>
+      <c r="L33" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A34" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="B34" t="s">
+        <v>3</v>
+      </c>
+      <c r="C34">
+        <v>2</v>
+      </c>
+      <c r="D34" t="s">
+        <v>244</v>
+      </c>
+      <c r="E34" t="s">
+        <v>4</v>
+      </c>
+      <c r="F34" s="2">
+        <v>43165</v>
+      </c>
+      <c r="G34" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H34" s="18">
+        <v>8</v>
+      </c>
+      <c r="I34" t="s">
+        <v>247</v>
+      </c>
+      <c r="J34" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>2.34</v>
+      </c>
+      <c r="K34" t="s">
+        <v>259</v>
+      </c>
+      <c r="L34" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A35" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="B35" t="s">
+        <v>3</v>
+      </c>
+      <c r="C35">
+        <v>2</v>
+      </c>
+      <c r="D35" t="s">
+        <v>244</v>
+      </c>
+      <c r="E35" t="s">
+        <v>4</v>
+      </c>
+      <c r="F35" s="2">
+        <v>43165</v>
+      </c>
+      <c r="G35" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H35" s="18">
+        <v>8</v>
+      </c>
+      <c r="I35" t="s">
+        <v>247</v>
+      </c>
+      <c r="J35" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>2.35</v>
+      </c>
+      <c r="K35" t="s">
+        <v>260</v>
+      </c>
+      <c r="L35" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A36" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="B36" t="s">
+        <v>3</v>
+      </c>
+      <c r="C36">
+        <v>2</v>
+      </c>
+      <c r="D36" t="s">
+        <v>244</v>
+      </c>
+      <c r="E36" t="s">
+        <v>4</v>
+      </c>
+      <c r="F36" s="2">
+        <v>43165</v>
+      </c>
+      <c r="G36" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H36" s="18">
+        <v>9</v>
+      </c>
+      <c r="I36" t="s">
+        <v>248</v>
+      </c>
+      <c r="J36" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>2.36</v>
+      </c>
+      <c r="K36" t="s">
+        <v>261</v>
+      </c>
+      <c r="L36" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A37" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="B37" t="s">
+        <v>3</v>
+      </c>
+      <c r="C37">
+        <v>2</v>
+      </c>
+      <c r="D37" t="s">
+        <v>244</v>
+      </c>
+      <c r="E37" t="s">
+        <v>4</v>
+      </c>
+      <c r="F37" s="2">
+        <v>43165</v>
+      </c>
+      <c r="G37" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H37" s="18">
+        <v>9</v>
+      </c>
+      <c r="I37" t="s">
+        <v>248</v>
+      </c>
+      <c r="J37" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>2.37</v>
+      </c>
+      <c r="K37" t="s">
+        <v>262</v>
+      </c>
+      <c r="L37" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A38" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="B38" t="s">
+        <v>3</v>
+      </c>
+      <c r="C38">
+        <v>2</v>
+      </c>
+      <c r="D38" t="s">
+        <v>244</v>
+      </c>
+      <c r="E38" t="s">
+        <v>4</v>
+      </c>
+      <c r="F38" s="2">
+        <v>43165</v>
+      </c>
+      <c r="G38" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H38" s="18">
+        <v>9</v>
+      </c>
+      <c r="I38" t="s">
+        <v>248</v>
+      </c>
+      <c r="J38" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>2.38</v>
+      </c>
+      <c r="K38" t="s">
+        <v>263</v>
+      </c>
+      <c r="L38" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A39" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="B39" t="s">
+        <v>3</v>
+      </c>
+      <c r="C39">
+        <v>2</v>
+      </c>
+      <c r="D39" t="s">
+        <v>244</v>
+      </c>
+      <c r="E39" t="s">
+        <v>4</v>
+      </c>
+      <c r="F39" s="2">
+        <v>43165</v>
+      </c>
+      <c r="G39" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H39" s="18">
+        <v>9</v>
+      </c>
+      <c r="I39" t="s">
+        <v>248</v>
+      </c>
+      <c r="J39" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>2.39</v>
+      </c>
+      <c r="K39" t="s">
+        <v>264</v>
+      </c>
+      <c r="L39" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="40" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A40" s="4" t="s">
+        <v>230</v>
+      </c>
+      <c r="B40" t="s">
+        <v>3</v>
+      </c>
+      <c r="C40">
+        <v>2</v>
+      </c>
+      <c r="D40" t="s">
+        <v>244</v>
+      </c>
+      <c r="E40" t="s">
+        <v>4</v>
+      </c>
+      <c r="F40" s="2">
+        <v>43165</v>
+      </c>
+      <c r="G40" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H40" s="18">
+        <v>9</v>
+      </c>
+      <c r="I40" t="s">
+        <v>248</v>
+      </c>
+      <c r="J40" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>2.40</v>
+      </c>
+      <c r="K40" t="s">
+        <v>265</v>
+      </c>
+      <c r="L40" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A41" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="B41" t="s">
+        <v>3</v>
+      </c>
+      <c r="C41">
+        <v>2</v>
+      </c>
+      <c r="D41" t="s">
+        <v>244</v>
+      </c>
+      <c r="E41" t="s">
+        <v>4</v>
+      </c>
+      <c r="F41" s="2">
+        <v>43165</v>
+      </c>
+      <c r="G41" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H41" s="18">
+        <v>9</v>
+      </c>
+      <c r="I41" t="s">
+        <v>248</v>
+      </c>
+      <c r="J41" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>2.41</v>
+      </c>
+      <c r="K41" t="s">
+        <v>278</v>
+      </c>
+      <c r="L41" t="s">
+        <v>203</v>
+      </c>
+      <c r="M41" s="2">
+        <v>43165</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A42" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="B42" t="s">
+        <v>3</v>
+      </c>
+      <c r="C42">
+        <v>2</v>
+      </c>
+      <c r="D42" t="s">
+        <v>244</v>
+      </c>
+      <c r="E42" t="s">
+        <v>4</v>
+      </c>
+      <c r="F42" s="2">
+        <v>43165</v>
+      </c>
+      <c r="G42" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H42" s="18">
+        <v>9</v>
+      </c>
+      <c r="I42" t="s">
+        <v>248</v>
+      </c>
+      <c r="J42" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>2.42</v>
+      </c>
+      <c r="K42" t="s">
+        <v>266</v>
+      </c>
+      <c r="L42" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A43" s="4" t="s">
+        <v>233</v>
+      </c>
+      <c r="B43" t="s">
+        <v>3</v>
+      </c>
+      <c r="C43">
+        <v>2</v>
+      </c>
+      <c r="D43" t="s">
+        <v>244</v>
+      </c>
+      <c r="E43" t="s">
+        <v>4</v>
+      </c>
+      <c r="F43" s="2">
+        <v>43165</v>
+      </c>
+      <c r="G43" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H43" s="18">
+        <v>9</v>
+      </c>
+      <c r="I43" t="s">
+        <v>248</v>
+      </c>
+      <c r="J43" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>2.43</v>
+      </c>
+      <c r="K43" t="s">
+        <v>267</v>
+      </c>
+      <c r="L43" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="44" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A44" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="B44" t="s">
+        <v>3</v>
+      </c>
+      <c r="C44">
+        <v>2</v>
+      </c>
+      <c r="D44" t="s">
+        <v>244</v>
+      </c>
+      <c r="E44" t="s">
+        <v>4</v>
+      </c>
+      <c r="F44" s="2">
+        <v>43165</v>
+      </c>
+      <c r="G44" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H44" s="18">
+        <v>9</v>
+      </c>
+      <c r="I44" t="s">
+        <v>248</v>
+      </c>
+      <c r="J44" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>2.44</v>
+      </c>
+      <c r="K44" t="s">
+        <v>268</v>
+      </c>
+      <c r="L44" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A45" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="B45" t="s">
+        <v>3</v>
+      </c>
+      <c r="C45">
+        <v>2</v>
+      </c>
+      <c r="D45" t="s">
+        <v>244</v>
+      </c>
+      <c r="E45" t="s">
+        <v>4</v>
+      </c>
+      <c r="F45" s="2">
+        <v>43165</v>
+      </c>
+      <c r="G45" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H45" s="18">
+        <v>9</v>
+      </c>
+      <c r="I45" t="s">
+        <v>248</v>
+      </c>
+      <c r="J45" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>2.45</v>
+      </c>
+      <c r="K45" t="s">
+        <v>269</v>
+      </c>
+      <c r="L45" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="46" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A46" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="B46" t="s">
+        <v>3</v>
+      </c>
+      <c r="C46">
+        <v>2</v>
+      </c>
+      <c r="D46" t="s">
+        <v>244</v>
+      </c>
+      <c r="E46" t="s">
+        <v>4</v>
+      </c>
+      <c r="F46" s="2">
+        <v>43165</v>
+      </c>
+      <c r="G46" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H46" s="18">
+        <v>9</v>
+      </c>
+      <c r="I46" t="s">
+        <v>248</v>
+      </c>
+      <c r="J46" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>2.46</v>
+      </c>
+      <c r="K46" t="s">
+        <v>270</v>
+      </c>
+      <c r="L46" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="47" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A47" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="B47" t="s">
+        <v>3</v>
+      </c>
+      <c r="C47">
+        <v>2</v>
+      </c>
+      <c r="D47" t="s">
+        <v>244</v>
+      </c>
+      <c r="E47" t="s">
+        <v>4</v>
+      </c>
+      <c r="F47" s="2">
+        <v>43165</v>
+      </c>
+      <c r="G47" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H47" s="18">
+        <v>9</v>
+      </c>
+      <c r="I47" t="s">
+        <v>248</v>
+      </c>
+      <c r="J47" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>2.47</v>
+      </c>
+      <c r="K47" t="s">
+        <v>271</v>
+      </c>
+      <c r="L47" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="48" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A48" s="4" t="s">
+        <v>238</v>
+      </c>
+      <c r="B48" t="s">
+        <v>3</v>
+      </c>
+      <c r="C48">
+        <v>2</v>
+      </c>
+      <c r="D48" t="s">
+        <v>244</v>
+      </c>
+      <c r="E48" t="s">
+        <v>4</v>
+      </c>
+      <c r="F48" s="2">
+        <v>43165</v>
+      </c>
+      <c r="G48" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H48" s="18">
+        <v>9</v>
+      </c>
+      <c r="I48" t="s">
+        <v>248</v>
+      </c>
+      <c r="J48" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>2.48</v>
+      </c>
+      <c r="K48" t="s">
+        <v>272</v>
+      </c>
+      <c r="L48" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A49" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="B49" t="s">
+        <v>3</v>
+      </c>
+      <c r="C49">
+        <v>2</v>
+      </c>
+      <c r="D49" t="s">
+        <v>244</v>
+      </c>
+      <c r="E49" t="s">
+        <v>4</v>
+      </c>
+      <c r="F49" s="2">
+        <v>43165</v>
+      </c>
+      <c r="G49" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H49" s="18">
+        <v>9</v>
+      </c>
+      <c r="I49" t="s">
+        <v>248</v>
+      </c>
+      <c r="J49" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>2.49</v>
+      </c>
+      <c r="K49" t="s">
+        <v>273</v>
+      </c>
+      <c r="L49" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A50" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="B50" t="s">
+        <v>3</v>
+      </c>
+      <c r="C50">
+        <v>2</v>
+      </c>
+      <c r="D50" t="s">
+        <v>244</v>
+      </c>
+      <c r="E50" t="s">
+        <v>4</v>
+      </c>
+      <c r="F50" s="2">
+        <v>43165</v>
+      </c>
+      <c r="G50" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H50" s="18">
+        <v>9</v>
+      </c>
+      <c r="I50" t="s">
+        <v>248</v>
+      </c>
+      <c r="J50" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>2.50</v>
+      </c>
+      <c r="K50" t="s">
+        <v>274</v>
+      </c>
+      <c r="L50" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A51" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="B51" t="s">
+        <v>3</v>
+      </c>
+      <c r="C51">
+        <v>2</v>
+      </c>
+      <c r="D51" t="s">
+        <v>244</v>
+      </c>
+      <c r="E51" t="s">
+        <v>4</v>
+      </c>
+      <c r="F51" s="2">
+        <v>43165</v>
+      </c>
+      <c r="G51" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H51" s="18">
+        <v>9</v>
+      </c>
+      <c r="I51" t="s">
+        <v>248</v>
+      </c>
+      <c r="J51" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>2.51</v>
+      </c>
+      <c r="K51" t="s">
+        <v>275</v>
+      </c>
+      <c r="L51" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="52" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A52" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="B52" t="s">
+        <v>3</v>
+      </c>
+      <c r="C52">
+        <v>2</v>
+      </c>
+      <c r="D52" t="s">
+        <v>244</v>
+      </c>
+      <c r="E52" t="s">
+        <v>4</v>
+      </c>
+      <c r="F52" s="2">
+        <v>43165</v>
+      </c>
+      <c r="G52" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H52" s="18">
+        <v>9</v>
+      </c>
+      <c r="I52" t="s">
+        <v>248</v>
+      </c>
+      <c r="J52" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>2.52</v>
+      </c>
+      <c r="K52" t="s">
+        <v>276</v>
+      </c>
+      <c r="L52" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="53" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A53" s="4" t="s">
+        <v>243</v>
+      </c>
+      <c r="B53" t="s">
+        <v>3</v>
+      </c>
+      <c r="C53">
+        <v>2</v>
+      </c>
+      <c r="D53" t="s">
+        <v>244</v>
+      </c>
+      <c r="E53" t="s">
+        <v>4</v>
+      </c>
+      <c r="F53" s="2">
+        <v>43165</v>
+      </c>
+      <c r="G53" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H53" s="18">
+        <v>9</v>
+      </c>
+      <c r="I53" t="s">
+        <v>248</v>
+      </c>
+      <c r="J53" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>2.53</v>
+      </c>
+      <c r="K53" t="s">
+        <v>277</v>
+      </c>
+      <c r="L53" t="s">
+        <v>206</v>
+      </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:M19">
-    <sortCondition ref="A2:A19"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:M20">
+    <sortCondition ref="A2:A20"/>
   </sortState>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
speciale tekens uit input verwijderd
</commit_message>
<xml_diff>
--- a/input/Bestandsbeschrijvingen.xlsx
+++ b/input/Bestandsbeschrijvingen.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ronaldkoenis/eclipse-workspace/maakmdto/input/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://regionaalarchiefnoordwestutrecht-my.sharepoint.com/personal/t_vorstenburg_regionaalarchiefnoordwestutrecht_nl/Documents/Bureaublad/Tijdelijk/maakmdto/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A026914F-354E-6241-A842-569DB7EC18DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{A026914F-354E-6241-A842-569DB7EC18DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{98B224CC-634F-4214-899C-12E31CDC3567}"/>
   <bookViews>
-    <workbookView xWindow="-16400" yWindow="-28200" windowWidth="51200" windowHeight="20220" xr2:uid="{597D6162-B0B0-3844-A8E7-90BC6507AED4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{597D6162-B0B0-3844-A8E7-90BC6507AED4}"/>
   </bookViews>
   <sheets>
     <sheet name="Bestand.zaak en doc" sheetId="1" r:id="rId1"/>
@@ -887,7 +887,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="6">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1407,22 +1407,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4C64E42-9F84-ED4B-87CF-18995B18C14B}">
   <dimension ref="A1:M53"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="140.1640625" customWidth="1"/>
+    <col min="1" max="1" width="140.125" customWidth="1"/>
     <col min="2" max="2" width="23" customWidth="1"/>
-    <col min="3" max="3" width="13.33203125" customWidth="1"/>
+    <col min="3" max="3" width="13.375" customWidth="1"/>
     <col min="4" max="4" width="37.5" customWidth="1"/>
-    <col min="5" max="7" width="10.83203125" customWidth="1"/>
-    <col min="8" max="8" width="10.83203125" style="18" customWidth="1"/>
-    <col min="9" max="9" width="39.33203125" customWidth="1"/>
-    <col min="10" max="10" width="9.83203125" customWidth="1"/>
-    <col min="11" max="11" width="111.6640625" customWidth="1"/>
-    <col min="12" max="12" width="28.6640625" customWidth="1"/>
-    <col min="13" max="13" width="20.83203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="10.875" customWidth="1"/>
+    <col min="8" max="8" width="12.375" style="18" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="39.375" customWidth="1"/>
+    <col min="10" max="10" width="9.875" customWidth="1"/>
+    <col min="11" max="11" width="77.625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="28.625" customWidth="1"/>
+    <col min="13" max="13" width="20.875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
         <v>8</v>
       </c>
@@ -1463,7 +1463,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:13">
       <c r="A2" s="4" t="s">
         <v>11</v>
       </c>
@@ -1501,7 +1501,7 @@
         <v>43046</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:13">
       <c r="A3" s="4" t="s">
         <v>10</v>
       </c>
@@ -1539,7 +1539,7 @@
         <v>43088</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:13">
       <c r="A4" s="4" t="s">
         <v>17</v>
       </c>
@@ -1579,7 +1579,7 @@
       </c>
       <c r="M4" s="2"/>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:13">
       <c r="A5" s="4" t="s">
         <v>24</v>
       </c>
@@ -1621,7 +1621,7 @@
         <v>43046</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:13">
       <c r="A6" s="4" t="s">
         <v>12</v>
       </c>
@@ -1663,7 +1663,7 @@
         <v>43046</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:13">
       <c r="A7" s="4" t="s">
         <v>14</v>
       </c>
@@ -1703,7 +1703,7 @@
       </c>
       <c r="M7" s="2"/>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:13">
       <c r="A8" s="4" t="s">
         <v>21</v>
       </c>
@@ -1743,7 +1743,7 @@
       </c>
       <c r="M8" s="2"/>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:13">
       <c r="A9" s="4" t="s">
         <v>15</v>
       </c>
@@ -1783,7 +1783,7 @@
       </c>
       <c r="M9" s="2"/>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:13">
       <c r="A10" s="4" t="s">
         <v>19</v>
       </c>
@@ -1823,7 +1823,7 @@
       </c>
       <c r="M10" s="2"/>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:13">
       <c r="A11" s="4" t="s">
         <v>18</v>
       </c>
@@ -1863,7 +1863,7 @@
       </c>
       <c r="M11" s="2"/>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:13">
       <c r="A12" s="4" t="s">
         <v>16</v>
       </c>
@@ -1903,7 +1903,7 @@
       </c>
       <c r="M12" s="2"/>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:13">
       <c r="A13" s="4" t="s">
         <v>25</v>
       </c>
@@ -1945,7 +1945,7 @@
         <v>43046</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:13">
       <c r="A14" s="4" t="s">
         <v>23</v>
       </c>
@@ -1987,7 +1987,7 @@
         <v>43046</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:13">
       <c r="A15" s="4" t="s">
         <v>20</v>
       </c>
@@ -2029,7 +2029,7 @@
         <v>43046</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:13">
       <c r="A16" s="4" t="s">
         <v>22</v>
       </c>
@@ -2071,7 +2071,7 @@
         <v>43046</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:13">
       <c r="A17" s="4" t="s">
         <v>26</v>
       </c>
@@ -2113,7 +2113,7 @@
         <v>43046</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:13">
       <c r="A18" s="4" t="s">
         <v>13</v>
       </c>
@@ -2153,7 +2153,7 @@
       </c>
       <c r="M18" s="2"/>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:13">
       <c r="A19" s="4" t="s">
         <v>212</v>
       </c>
@@ -2189,7 +2189,7 @@
         <v>43165</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:13">
       <c r="A20" s="4" t="s">
         <v>210</v>
       </c>
@@ -2225,7 +2225,7 @@
         <v>43165</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:13">
       <c r="A21" s="4" t="s">
         <v>211</v>
       </c>
@@ -2261,7 +2261,7 @@
         <v>43165</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:13">
       <c r="A22" s="4" t="s">
         <v>213</v>
       </c>
@@ -2303,7 +2303,7 @@
         <v>43165</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:13">
       <c r="A23" s="4" t="s">
         <v>214</v>
       </c>
@@ -2345,7 +2345,7 @@
         <v>43165</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:13">
       <c r="A24" s="4" t="s">
         <v>215</v>
       </c>
@@ -2387,7 +2387,7 @@
         <v>43165</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:13">
       <c r="A25" s="4" t="s">
         <v>216</v>
       </c>
@@ -2426,7 +2426,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:13">
       <c r="A26" s="4" t="s">
         <v>217</v>
       </c>
@@ -2465,7 +2465,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:13">
       <c r="A27" s="4" t="s">
         <v>218</v>
       </c>
@@ -2504,7 +2504,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:13">
       <c r="A28" s="4" t="s">
         <v>219</v>
       </c>
@@ -2543,7 +2543,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:13">
       <c r="A29" s="4" t="s">
         <v>220</v>
       </c>
@@ -2582,7 +2582,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:13">
       <c r="A30" s="4" t="s">
         <v>221</v>
       </c>
@@ -2621,7 +2621,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:13">
       <c r="A31" s="4" t="s">
         <v>222</v>
       </c>
@@ -2660,7 +2660,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:13">
       <c r="A32" s="4" t="s">
         <v>223</v>
       </c>
@@ -2702,7 +2702,7 @@
         <v>43165</v>
       </c>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:13">
       <c r="A33" s="4" t="s">
         <v>224</v>
       </c>
@@ -2741,7 +2741,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:13">
       <c r="A34" s="4" t="s">
         <v>225</v>
       </c>
@@ -2780,7 +2780,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:13">
       <c r="A35" s="4" t="s">
         <v>226</v>
       </c>
@@ -2819,7 +2819,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:13">
       <c r="A36" s="4" t="s">
         <v>227</v>
       </c>
@@ -2858,7 +2858,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:13">
       <c r="A37" s="4" t="s">
         <v>228</v>
       </c>
@@ -2897,7 +2897,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:13">
       <c r="A38" s="4" t="s">
         <v>229</v>
       </c>
@@ -2936,7 +2936,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:13">
       <c r="A39" s="4" t="s">
         <v>279</v>
       </c>
@@ -2975,7 +2975,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:13">
       <c r="A40" s="4" t="s">
         <v>230</v>
       </c>
@@ -3014,7 +3014,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:13">
       <c r="A41" s="4" t="s">
         <v>231</v>
       </c>
@@ -3056,7 +3056,7 @@
         <v>43165</v>
       </c>
     </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:13">
       <c r="A42" s="4" t="s">
         <v>232</v>
       </c>
@@ -3095,7 +3095,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:13">
       <c r="A43" s="4" t="s">
         <v>233</v>
       </c>
@@ -3134,7 +3134,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:13">
       <c r="A44" s="4" t="s">
         <v>234</v>
       </c>
@@ -3173,7 +3173,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:13">
       <c r="A45" s="4" t="s">
         <v>235</v>
       </c>
@@ -3212,7 +3212,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:13">
       <c r="A46" s="4" t="s">
         <v>236</v>
       </c>
@@ -3251,7 +3251,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:13">
       <c r="A47" s="4" t="s">
         <v>237</v>
       </c>
@@ -3290,7 +3290,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:13">
       <c r="A48" s="4" t="s">
         <v>238</v>
       </c>
@@ -3329,7 +3329,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:12">
       <c r="A49" s="4" t="s">
         <v>239</v>
       </c>
@@ -3368,7 +3368,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:12">
       <c r="A50" s="4" t="s">
         <v>240</v>
       </c>
@@ -3407,7 +3407,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:12">
       <c r="A51" s="4" t="s">
         <v>241</v>
       </c>
@@ -3446,7 +3446,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:12">
       <c r="A52" s="4" t="s">
         <v>242</v>
       </c>
@@ -3485,7 +3485,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:12">
       <c r="A53" s="4" t="s">
         <v>243</v>
       </c>
@@ -3536,15 +3536,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F695ACD-0E20-9446-8CA5-3DAED1E6C2C8}">
   <dimension ref="A1:C75"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="1" width="11" style="7" customWidth="1"/>
-    <col min="2" max="2" width="41.83203125" style="7" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="42.1640625" style="7" customWidth="1"/>
-    <col min="4" max="16384" width="10.83203125" style="7"/>
+    <col min="2" max="2" width="41.875" style="7" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="42.125" style="7" customWidth="1"/>
+    <col min="4" max="16384" width="10.875" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3">
       <c r="A1" s="7" t="s">
         <v>182</v>
       </c>
@@ -3555,7 +3555,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3">
       <c r="A2" s="5" t="s">
         <v>34</v>
       </c>
@@ -3563,7 +3563,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3">
       <c r="A3" s="8" t="s">
         <v>36</v>
       </c>
@@ -3571,7 +3571,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3">
       <c r="A4" s="8" t="s">
         <v>38</v>
       </c>
@@ -3579,7 +3579,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3">
       <c r="A5" s="8" t="s">
         <v>40</v>
       </c>
@@ -3587,7 +3587,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3">
       <c r="A6" s="8" t="s">
         <v>42</v>
       </c>
@@ -3595,7 +3595,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3">
       <c r="A7" s="8" t="s">
         <v>44</v>
       </c>
@@ -3603,7 +3603,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3">
       <c r="A8" s="8" t="s">
         <v>46</v>
       </c>
@@ -3611,7 +3611,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3">
       <c r="A9" s="8" t="s">
         <v>48</v>
       </c>
@@ -3619,7 +3619,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3">
       <c r="A10" s="8" t="s">
         <v>50</v>
       </c>
@@ -3627,7 +3627,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:3">
       <c r="A11" s="8" t="s">
         <v>52</v>
       </c>
@@ -3635,7 +3635,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:3">
       <c r="A12" s="8" t="s">
         <v>54</v>
       </c>
@@ -3643,7 +3643,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:3">
       <c r="A13" s="8" t="s">
         <v>56</v>
       </c>
@@ -3651,7 +3651,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:3">
       <c r="A14" s="8" t="s">
         <v>58</v>
       </c>
@@ -3659,7 +3659,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:3">
       <c r="A15" s="8" t="s">
         <v>60</v>
       </c>
@@ -3667,7 +3667,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:3">
       <c r="A16" s="8" t="s">
         <v>62</v>
       </c>
@@ -3675,7 +3675,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:2">
       <c r="A17" s="8" t="s">
         <v>64</v>
       </c>
@@ -3683,7 +3683,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:2">
       <c r="A18" s="8" t="s">
         <v>66</v>
       </c>
@@ -3691,7 +3691,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:2">
       <c r="A19" s="8" t="s">
         <v>68</v>
       </c>
@@ -3699,7 +3699,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:2">
       <c r="A20" s="8" t="s">
         <v>70</v>
       </c>
@@ -3707,7 +3707,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:2">
       <c r="A21" s="8" t="s">
         <v>72</v>
       </c>
@@ -3715,7 +3715,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:2">
       <c r="A22" s="8" t="s">
         <v>74</v>
       </c>
@@ -3723,7 +3723,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:2">
       <c r="A23" s="8" t="s">
         <v>76</v>
       </c>
@@ -3731,7 +3731,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:2">
       <c r="A24" s="8" t="s">
         <v>78</v>
       </c>
@@ -3739,7 +3739,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:2">
       <c r="A25" s="8" t="s">
         <v>80</v>
       </c>
@@ -3747,7 +3747,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:2">
       <c r="A26" s="8" t="s">
         <v>82</v>
       </c>
@@ -3755,7 +3755,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:2">
       <c r="A27" s="8" t="s">
         <v>84</v>
       </c>
@@ -3763,7 +3763,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:2">
       <c r="A28" s="8" t="s">
         <v>86</v>
       </c>
@@ -3771,7 +3771,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:2">
       <c r="A29" s="8" t="s">
         <v>88</v>
       </c>
@@ -3779,7 +3779,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:2">
       <c r="A30" s="8" t="s">
         <v>90</v>
       </c>
@@ -3787,7 +3787,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:2">
       <c r="A31" s="8" t="s">
         <v>92</v>
       </c>
@@ -3795,7 +3795,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:2">
       <c r="A32" s="8" t="s">
         <v>94</v>
       </c>
@@ -3803,7 +3803,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:2">
       <c r="A33" s="8" t="s">
         <v>96</v>
       </c>
@@ -3811,7 +3811,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:2">
       <c r="A34" s="8" t="s">
         <v>98</v>
       </c>
@@ -3819,7 +3819,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:2">
       <c r="A35" s="8" t="s">
         <v>100</v>
       </c>
@@ -3827,7 +3827,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:2">
       <c r="A36" s="8" t="s">
         <v>102</v>
       </c>
@@ -3835,7 +3835,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:2">
       <c r="A37" s="8" t="s">
         <v>104</v>
       </c>
@@ -3843,7 +3843,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:2">
       <c r="A38" s="8" t="s">
         <v>106</v>
       </c>
@@ -3851,7 +3851,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:2">
       <c r="A39" s="8" t="s">
         <v>108</v>
       </c>
@@ -3859,7 +3859,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:2">
       <c r="A40" s="8" t="s">
         <v>110</v>
       </c>
@@ -3867,7 +3867,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:2">
       <c r="A41" s="8" t="s">
         <v>112</v>
       </c>
@@ -3875,7 +3875,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:2">
       <c r="A42" s="8" t="s">
         <v>114</v>
       </c>
@@ -3883,7 +3883,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:2">
       <c r="A43" s="8" t="s">
         <v>116</v>
       </c>
@@ -3891,7 +3891,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:2">
       <c r="A44" s="8" t="s">
         <v>118</v>
       </c>
@@ -3899,7 +3899,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:2">
       <c r="A45" s="8" t="s">
         <v>120</v>
       </c>
@@ -3907,7 +3907,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:2">
       <c r="A46" s="8" t="s">
         <v>122</v>
       </c>
@@ -3915,7 +3915,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:2">
       <c r="A47" s="8" t="s">
         <v>124</v>
       </c>
@@ -3923,7 +3923,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:2">
       <c r="A48" s="8" t="s">
         <v>126</v>
       </c>
@@ -3931,7 +3931,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:2">
       <c r="A49" s="8" t="s">
         <v>128</v>
       </c>
@@ -3939,7 +3939,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:2">
       <c r="A50" s="8" t="s">
         <v>130</v>
       </c>
@@ -3947,7 +3947,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:2">
       <c r="A51" s="8" t="s">
         <v>132</v>
       </c>
@@ -3955,7 +3955,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:2">
       <c r="A52" s="8" t="s">
         <v>134</v>
       </c>
@@ -3963,7 +3963,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:2">
       <c r="A53" s="8" t="s">
         <v>136</v>
       </c>
@@ -3971,7 +3971,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:2">
       <c r="A54" s="8" t="s">
         <v>138</v>
       </c>
@@ -3979,7 +3979,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:2">
       <c r="A55" s="8" t="s">
         <v>140</v>
       </c>
@@ -3987,7 +3987,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:2">
       <c r="A56" s="8" t="s">
         <v>142</v>
       </c>
@@ -3995,7 +3995,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:2">
       <c r="A57" s="8" t="s">
         <v>144</v>
       </c>
@@ -4003,7 +4003,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:2">
       <c r="A58" s="8" t="s">
         <v>146</v>
       </c>
@@ -4011,7 +4011,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:2">
       <c r="A59" s="8" t="s">
         <v>148</v>
       </c>
@@ -4019,7 +4019,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:2">
       <c r="A60" s="8" t="s">
         <v>150</v>
       </c>
@@ -4027,7 +4027,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:2">
       <c r="A61" s="8" t="s">
         <v>152</v>
       </c>
@@ -4035,7 +4035,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:2">
       <c r="A62" s="8" t="s">
         <v>154</v>
       </c>
@@ -4043,7 +4043,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:2">
       <c r="A63" s="8" t="s">
         <v>156</v>
       </c>
@@ -4051,7 +4051,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:2">
       <c r="A64" s="8" t="s">
         <v>158</v>
       </c>
@@ -4059,7 +4059,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:2">
       <c r="A65" s="8" t="s">
         <v>160</v>
       </c>
@@ -4067,7 +4067,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:2">
       <c r="A66" s="8" t="s">
         <v>162</v>
       </c>
@@ -4075,7 +4075,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:2">
       <c r="A67" s="8" t="s">
         <v>164</v>
       </c>
@@ -4083,7 +4083,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:2">
       <c r="A68" s="8" t="s">
         <v>166</v>
       </c>
@@ -4091,7 +4091,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:2">
       <c r="A69" s="8" t="s">
         <v>168</v>
       </c>
@@ -4099,7 +4099,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:2">
       <c r="A70" s="8" t="s">
         <v>170</v>
       </c>
@@ -4107,7 +4107,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:2">
       <c r="A71" s="8" t="s">
         <v>172</v>
       </c>
@@ -4115,7 +4115,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:2">
       <c r="A72" s="13" t="s">
         <v>174</v>
       </c>
@@ -4123,7 +4123,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:2">
       <c r="A73" s="5" t="s">
         <v>176</v>
       </c>
@@ -4131,7 +4131,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:2">
       <c r="A74" s="8" t="s">
         <v>178</v>
       </c>
@@ -4139,7 +4139,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:2">
       <c r="A75" s="13" t="s">
         <v>180</v>
       </c>
@@ -4155,12 +4155,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA278A34-3380-8A44-8E5C-29BA0CE91D7C}">
   <dimension ref="A2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="93.6640625" customWidth="1"/>
+    <col min="1" max="1" width="93.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:1">
       <c r="A2" t="s">
         <v>0</v>
       </c>

</xml_diff>